<commit_message>
feat(onvio): add gestta validation and update service requests
</commit_message>
<xml_diff>
--- a/Unecont/assets/templates/empresas-template.xlsx
+++ b/Unecont/assets/templates/empresas-template.xlsx
@@ -397,7 +397,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:I3"/>
+  <dimension ref="A1:L3"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -427,6 +427,15 @@
       <c r="I1" t="str">
         <v>ARQUIVOS</v>
       </c>
+      <c r="J1" t="str">
+        <v>ONVIO_CLIENT_ID</v>
+      </c>
+      <c r="K1" t="str">
+        <v>ONVIO_REQUESTER_ID</v>
+      </c>
+      <c r="L1" t="str">
+        <v>ONVIO_DEPARTMENT_ID</v>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="str">
@@ -456,6 +465,15 @@
       <c r="I2" t="str">
         <v>Empresa 1 - Relatorio A.pdf; Empresa 1 - Relatorio B.xlsx</v>
       </c>
+      <c r="J2" t="str">
+        <v/>
+      </c>
+      <c r="K2" t="str">
+        <v/>
+      </c>
+      <c r="L2" t="str">
+        <v/>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="str">
@@ -485,10 +503,19 @@
       <c r="I3" t="str">
         <v/>
       </c>
+      <c r="J3" t="str">
+        <v/>
+      </c>
+      <c r="K3" t="str">
+        <v/>
+      </c>
+      <c r="L3" t="str">
+        <v/>
+      </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:I3"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:L3"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>